<commit_message>
Data: Push user's updated Excel sheet containing Mentor Email mappings
</commit_message>
<xml_diff>
--- a/Course wise Mentor Skillset map.xlsx
+++ b/Course wise Mentor Skillset map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://theinnovationstory-my.sharepoint.com/personal/abinash_dash_theinnovationstory_com/Documents/Desktop/Antigravity/Calendar scheduling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="8_{033DB306-5DC3-4C71-9582-C90156F962C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49182BF3-56C5-4418-BF55-124F8D24E7B9}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{033DB306-5DC3-4C71-9582-C90156F962C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71018F02-A7D8-454E-AA71-97FCF2C5CD69}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{01402C56-8DF7-465C-BE20-9C72B5E82270}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{01402C56-8DF7-465C-BE20-9C72B5E82270}"/>
   </bookViews>
   <sheets>
     <sheet name="Dadar" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Bandra!$A$1:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Dadar!$A$1:$L$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mentor shifts'!$A$1:$D$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mentor shifts'!$A$1:$E$32</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="145">
   <si>
     <t>Course Name</t>
   </si>
@@ -383,6 +383,102 @@
   </si>
   <si>
     <t>Christmas</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>akshat.shah@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>janhavi@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>ayushi.lowanshi@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>ayush.dwivedy@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>gaurish.vaze@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>vaishnavi.bodke@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>anuj.rathod@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>jaykumar.patel@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>latifa@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>rui.jadhav@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>saiyad.husain@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>aniruddh.iyer@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>saket.singh@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>karan.jain@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>anthony.dsouza@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>aniket.karkala@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>ankit.chheda@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>vedant.patel@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>om.kulkarni@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>mayuresh.patil@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>yash.prajapati@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>dhruval.vachhani@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>drashti.shah@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>utkarsh.kankaria@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>siddhesh.murudkar@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>vedant.raut@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>mayur.gosavi@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>shashank.ganvir@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>lavkush.chaudhary@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>shashank@theinnovationstory.com</t>
+  </si>
+  <si>
+    <t>rohan.gaikwad@theinnovationstory.com</t>
   </si>
 </sst>
 </file>
@@ -1515,10 +1611,10 @@
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="A24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2027,467 +2123,564 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DC41263-2F85-4A05-8006-4010FB9DE498}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.90625" customWidth="1"/>
-    <col min="2" max="2" width="9.453125" customWidth="1"/>
-    <col min="3" max="3" width="33.81640625" customWidth="1"/>
-    <col min="4" max="4" width="47.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" customWidth="1"/>
+    <col min="4" max="4" width="33.81640625" customWidth="1"/>
+    <col min="5" max="5" width="47.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
         <v>69</v>
       </c>
       <c r="B1" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="D1" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="E1" s="19" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>67</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="D28" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>79</v>
+      <c r="B31" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>79</v>
       </c>
       <c r="D31" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="E32" s="3" t="s">
         <v>82</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D32" xr:uid="{2DC41263-2F85-4A05-8006-4010FB9DE498}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D32">
-      <sortCondition ref="C1:C32"/>
+  <autoFilter ref="A1:E32" xr:uid="{2DC41263-2F85-4A05-8006-4010FB9DE498}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E32">
+      <sortCondition ref="D1:D32"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>